<commit_message>
Publish Ivrea_2016_WC, Ivrea_2017_WC, Ivrea_2024_WC, LaSeu_2017_WC
</commit_message>
<xml_diff>
--- a/events/Ivrea_2016_WC/Ivrea_2016_WC_start.xlsx
+++ b/events/Ivrea_2016_WC/Ivrea_2016_WC_start.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W504"/>
+  <dimension ref="A1:AC504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,17 +519,47 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
+          <t>Name4</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Name5</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Name6</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
           <t>ICF_ID1</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>ICF_ID2</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>ICF_ID3</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>ICF_ID4</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>ICF_ID5</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>ICF_ID6</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1307,7 @@
           <t>ROSSI Lucas</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr">
+      <c r="X16" t="inlineStr">
         <is>
           <t>36925</t>
         </is>
@@ -1335,7 +1365,7 @@
           <t>MARZO Daniel</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr">
+      <c r="X17" t="inlineStr">
         <is>
           <t>35757</t>
         </is>
@@ -1393,7 +1423,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="X18" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -1451,7 +1481,7 @@
           <t>SHU Jianming</t>
         </is>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="X19" t="inlineStr">
         <is>
           <t>47327</t>
         </is>
@@ -1509,7 +1539,7 @@
           <t>DOBY Mathieu</t>
         </is>
       </c>
-      <c r="U20" t="inlineStr">
+      <c r="X20" t="inlineStr">
         <is>
           <t>35292</t>
         </is>
@@ -1567,7 +1597,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="X21" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -1625,7 +1655,7 @@
           <t>SMITH Tyler</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="X22" t="inlineStr">
         <is>
           <t>51904</t>
         </is>
@@ -1683,7 +1713,7 @@
           <t>JEKLIN Jakob</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="X23" t="inlineStr">
         <is>
           <t>42022</t>
         </is>
@@ -1741,7 +1771,7 @@
           <t>COF Blaz</t>
         </is>
       </c>
-      <c r="U24" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>36897</t>
         </is>
@@ -1799,7 +1829,7 @@
           <t>SOSA Angelo</t>
         </is>
       </c>
-      <c r="U25" t="inlineStr">
+      <c r="X25" t="inlineStr">
         <is>
           <t>51793</t>
         </is>
@@ -1857,7 +1887,7 @@
           <t>WASHER Patrick</t>
         </is>
       </c>
-      <c r="U26" t="inlineStr">
+      <c r="X26" t="inlineStr">
         <is>
           <t>42081</t>
         </is>
@@ -1915,7 +1945,7 @@
           <t>SILVA Jose</t>
         </is>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="X27" t="inlineStr">
         <is>
           <t>36494</t>
         </is>
@@ -1973,7 +2003,7 @@
           <t>CORREA Charles</t>
         </is>
       </c>
-      <c r="U28" t="inlineStr">
+      <c r="X28" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
@@ -2031,7 +2061,7 @@
           <t>PARES Lluis</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="X29" t="inlineStr">
         <is>
           <t>44008</t>
         </is>
@@ -2089,7 +2119,7 @@
           <t>GIBB Benjamin</t>
         </is>
       </c>
-      <c r="U30" t="inlineStr">
+      <c r="X30" t="inlineStr">
         <is>
           <t>36711</t>
         </is>
@@ -2147,7 +2177,7 @@
           <t>CHEN Fangjia</t>
         </is>
       </c>
-      <c r="U31" t="inlineStr">
+      <c r="X31" t="inlineStr">
         <is>
           <t>42638</t>
         </is>
@@ -2205,7 +2235,7 @@
           <t>CURCEL Leonardo</t>
         </is>
       </c>
-      <c r="U32" t="inlineStr">
+      <c r="X32" t="inlineStr">
         <is>
           <t>38014</t>
         </is>
@@ -2263,7 +2293,7 @@
           <t>GARMENDIA Aitor</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="X33" t="inlineStr">
         <is>
           <t>35745</t>
         </is>
@@ -2374,7 +2404,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="X35" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -2432,7 +2462,7 @@
           <t>CECCON Paolo</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="X36" t="inlineStr">
         <is>
           <t>39903</t>
         </is>
@@ -2490,7 +2520,7 @@
           <t>MIRGORODSKY Marko</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="X37" t="inlineStr">
         <is>
           <t>42019</t>
         </is>
@@ -2548,7 +2578,7 @@
           <t>JEGOU Liam</t>
         </is>
       </c>
-      <c r="U38" t="inlineStr">
+      <c r="X38" t="inlineStr">
         <is>
           <t>35820</t>
         </is>
@@ -2606,7 +2636,7 @@
           <t>FOULON Kilian</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="X39" t="inlineStr">
         <is>
           <t>35602</t>
         </is>
@@ -2664,7 +2694,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="X40" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -2722,7 +2752,7 @@
           <t>SMEDLEY Cameron</t>
         </is>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="X41" t="inlineStr">
         <is>
           <t>35543</t>
         </is>
@@ -2780,7 +2810,7 @@
           <t>JANE Michal</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="X42" t="inlineStr">
         <is>
           <t>35059</t>
         </is>
@@ -2838,7 +2868,7 @@
           <t>BORROWS Ian</t>
         </is>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="X43" t="inlineStr">
         <is>
           <t>36534</t>
         </is>
@@ -2896,7 +2926,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="X44" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -2954,7 +2984,7 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="X45" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -3012,7 +3042,7 @@
           <t>BURGESS Adam</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="X46" t="inlineStr">
         <is>
           <t>35647</t>
         </is>
@@ -3070,7 +3100,7 @@
           <t>THOMAS Martin</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="X47" t="inlineStr">
         <is>
           <t>35412</t>
         </is>
@@ -3128,7 +3158,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U48" t="inlineStr">
+      <c r="X48" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -3292,7 +3322,7 @@
           <t>PESCHIER Nicolas</t>
         </is>
       </c>
-      <c r="U51" t="inlineStr">
+      <c r="X51" t="inlineStr">
         <is>
           <t>35401</t>
         </is>
@@ -3350,7 +3380,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U52" t="inlineStr">
+      <c r="X52" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -3408,7 +3438,7 @@
           <t>WESTLEY Ryan</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="X53" t="inlineStr">
         <is>
           <t>35651</t>
         </is>
@@ -3466,7 +3496,7 @@
           <t>CIPRESSI Stefano</t>
         </is>
       </c>
-      <c r="U54" t="inlineStr">
+      <c r="X54" t="inlineStr">
         <is>
           <t>35495</t>
         </is>
@@ -3524,7 +3554,7 @@
           <t>TILLARD Pierre-Antoine</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="X55" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
@@ -3582,7 +3612,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U56" t="inlineStr">
+      <c r="X56" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -3640,7 +3670,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr">
+      <c r="X57" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -3698,7 +3728,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U58" t="inlineStr">
+      <c r="X58" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -3756,7 +3786,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
+      <c r="X59" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -3814,7 +3844,7 @@
           <t>HENRY Margaux</t>
         </is>
       </c>
-      <c r="U60" t="inlineStr">
+      <c r="X60" t="inlineStr">
         <is>
           <t>51995</t>
         </is>
@@ -3872,7 +3902,7 @@
           <t>NAVEAU Laurine</t>
         </is>
       </c>
-      <c r="U61" t="inlineStr">
+      <c r="X61" t="inlineStr">
         <is>
           <t>53246</t>
         </is>
@@ -3930,7 +3960,7 @@
           <t>GLEJTEKOVA Simona</t>
         </is>
       </c>
-      <c r="U62" t="inlineStr">
+      <c r="X62" t="inlineStr">
         <is>
           <t>55166</t>
         </is>
@@ -3988,7 +4018,7 @@
           <t>SKACHOVA Monika</t>
         </is>
       </c>
-      <c r="U63" t="inlineStr">
+      <c r="X63" t="inlineStr">
         <is>
           <t>53078</t>
         </is>
@@ -4046,7 +4076,7 @@
           <t>MACEKOVA Simona</t>
         </is>
       </c>
-      <c r="U64" t="inlineStr">
+      <c r="X64" t="inlineStr">
         <is>
           <t>45153</t>
         </is>
@@ -4157,7 +4187,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U66" t="inlineStr">
+      <c r="X66" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -4215,7 +4245,7 @@
           <t>DANIELS Haley</t>
         </is>
       </c>
-      <c r="U67" t="inlineStr">
+      <c r="X67" t="inlineStr">
         <is>
           <t>36260</t>
         </is>
@@ -4273,7 +4303,7 @@
           <t>BIZJAK Nina</t>
         </is>
       </c>
-      <c r="U68" t="inlineStr">
+      <c r="X68" t="inlineStr">
         <is>
           <t>39984</t>
         </is>
@@ -4331,7 +4361,7 @@
           <t>RANKIN Georgia</t>
         </is>
       </c>
-      <c r="U69" t="inlineStr">
+      <c r="X69" t="inlineStr">
         <is>
           <t>38435</t>
         </is>
@@ -4389,7 +4419,7 @@
           <t>MATULKOVA Jana</t>
         </is>
       </c>
-      <c r="U70" t="inlineStr">
+      <c r="X70" t="inlineStr">
         <is>
           <t>37274</t>
         </is>
@@ -4447,7 +4477,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U71" t="inlineStr">
+      <c r="X71" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -4505,7 +4535,7 @@
           <t>TIXIER Cecile</t>
         </is>
       </c>
-      <c r="U72" t="inlineStr">
+      <c r="X72" t="inlineStr">
         <is>
           <t>35687</t>
         </is>
@@ -4563,7 +4593,7 @@
           <t>JACQUET Claire</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr">
+      <c r="X73" t="inlineStr">
         <is>
           <t>35684</t>
         </is>
@@ -4621,7 +4651,7 @@
           <t>BORROWS Alison</t>
         </is>
       </c>
-      <c r="U74" t="inlineStr">
+      <c r="X74" t="inlineStr">
         <is>
           <t>38440</t>
         </is>
@@ -4679,7 +4709,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U75" t="inlineStr">
+      <c r="X75" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -4737,7 +4767,7 @@
           <t>WERATSCHNIG Nadine</t>
         </is>
       </c>
-      <c r="U76" t="inlineStr">
+      <c r="X76" t="inlineStr">
         <is>
           <t>41613</t>
         </is>
@@ -4795,7 +4825,7 @@
           <t>LAZKANO Miren</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr">
+      <c r="X77" t="inlineStr">
         <is>
           <t>35748</t>
         </is>
@@ -4906,7 +4936,7 @@
           <t>GIBSON Eilidh</t>
         </is>
       </c>
-      <c r="U79" t="inlineStr">
+      <c r="X79" t="inlineStr">
         <is>
           <t>36708</t>
         </is>
@@ -4964,7 +4994,7 @@
           <t>JANCOVA Monika</t>
         </is>
       </c>
-      <c r="U80" t="inlineStr">
+      <c r="X80" t="inlineStr">
         <is>
           <t>36015</t>
         </is>
@@ -5022,7 +5052,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U81" t="inlineStr">
+      <c r="X81" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -5080,7 +5110,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U82" t="inlineStr">
+      <c r="X82" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -5138,7 +5168,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U83" t="inlineStr">
+      <c r="X83" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -5196,7 +5226,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U84" t="inlineStr">
+      <c r="X84" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -5254,7 +5284,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U85" t="inlineStr">
+      <c r="X85" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -5312,7 +5342,7 @@
           <t>SOARES Renan</t>
         </is>
       </c>
-      <c r="U86" t="inlineStr">
+      <c r="X86" t="inlineStr">
         <is>
           <t>42776</t>
         </is>
@@ -5423,7 +5453,7 @@
           <t>AKINYEMI Johnathan</t>
         </is>
       </c>
-      <c r="U88" t="inlineStr">
+      <c r="X88" t="inlineStr">
         <is>
           <t>36822</t>
         </is>
@@ -5534,7 +5564,7 @@
           <t>LEE EDWARDS Ciaran</t>
         </is>
       </c>
-      <c r="U90" t="inlineStr">
+      <c r="X90" t="inlineStr">
         <is>
           <t>35614</t>
         </is>
@@ -5592,7 +5622,7 @@
           <t>SWETNAM Huw</t>
         </is>
       </c>
-      <c r="U91" t="inlineStr">
+      <c r="X91" t="inlineStr">
         <is>
           <t>35652</t>
         </is>
@@ -5650,7 +5680,7 @@
           <t>DRAPER Warwick</t>
         </is>
       </c>
-      <c r="U92" t="inlineStr">
+      <c r="X92" t="inlineStr">
         <is>
           <t>36536</t>
         </is>
@@ -5708,7 +5738,7 @@
           <t>WESTFALL Tyler</t>
         </is>
       </c>
-      <c r="U93" t="inlineStr">
+      <c r="X93" t="inlineStr">
         <is>
           <t>51919</t>
         </is>
@@ -5766,7 +5796,7 @@
           <t>MAPELLI Guilherme Marcello</t>
         </is>
       </c>
-      <c r="U94" t="inlineStr">
+      <c r="X94" t="inlineStr">
         <is>
           <t>38015</t>
         </is>
@@ -5824,7 +5854,7 @@
           <t>OGURA Takashi</t>
         </is>
       </c>
-      <c r="U95" t="inlineStr">
+      <c r="X95" t="inlineStr">
         <is>
           <t>37679</t>
         </is>
@@ -5882,7 +5912,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U96" t="inlineStr">
+      <c r="X96" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -5940,7 +5970,7 @@
           <t>WEGER Jakob</t>
         </is>
       </c>
-      <c r="U97" t="inlineStr">
+      <c r="X97" t="inlineStr">
         <is>
           <t>54909</t>
         </is>
@@ -5998,7 +6028,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U98" t="inlineStr">
+      <c r="X98" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -6056,7 +6086,7 @@
           <t>SMITH Tyler</t>
         </is>
       </c>
-      <c r="U99" t="inlineStr">
+      <c r="X99" t="inlineStr">
         <is>
           <t>51904</t>
         </is>
@@ -6114,7 +6144,7 @@
           <t>QUAN Xin</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr">
+      <c r="X100" t="inlineStr">
         <is>
           <t>62343</t>
         </is>
@@ -6172,7 +6202,7 @@
           <t>CORTEZ Geronimo</t>
         </is>
       </c>
-      <c r="U101" t="inlineStr">
+      <c r="X101" t="inlineStr">
         <is>
           <t>51835</t>
         </is>
@@ -6230,7 +6260,7 @@
           <t>CHIARELLO Gelindo</t>
         </is>
       </c>
-      <c r="U102" t="inlineStr">
+      <c r="X102" t="inlineStr">
         <is>
           <t>39956</t>
         </is>
@@ -6288,7 +6318,7 @@
           <t>PEREZ Alexis</t>
         </is>
       </c>
-      <c r="U103" t="inlineStr">
+      <c r="X103" t="inlineStr">
         <is>
           <t>41649</t>
         </is>
@@ -6346,7 +6376,7 @@
           <t>ROSSI Lucas</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr">
+      <c r="X104" t="inlineStr">
         <is>
           <t>36925</t>
         </is>
@@ -6404,7 +6434,7 @@
           <t>MARTINS TAQUES Ricardo</t>
         </is>
       </c>
-      <c r="U105" t="inlineStr">
+      <c r="X105" t="inlineStr">
         <is>
           <t>38022</t>
         </is>
@@ -6462,7 +6492,7 @@
           <t>MARTIN Gerome</t>
         </is>
       </c>
-      <c r="U106" t="inlineStr">
+      <c r="X106" t="inlineStr">
         <is>
           <t>36720</t>
         </is>
@@ -6520,7 +6550,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U107" t="inlineStr">
+      <c r="X107" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -6578,7 +6608,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U108" t="inlineStr">
+      <c r="X108" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -6636,7 +6666,7 @@
           <t>TAN Ya</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr">
+      <c r="X109" t="inlineStr">
         <is>
           <t>52024</t>
         </is>
@@ -6694,7 +6724,7 @@
           <t>SCHLAEFLI Jeremias</t>
         </is>
       </c>
-      <c r="U110" t="inlineStr">
+      <c r="X110" t="inlineStr">
         <is>
           <t>35430</t>
         </is>
@@ -6752,7 +6782,7 @@
           <t>BUTCHER Finn</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
+      <c r="X111" t="inlineStr">
         <is>
           <t>36663</t>
         </is>
@@ -6810,7 +6840,7 @@
           <t>TSVIET Igor</t>
         </is>
       </c>
-      <c r="U112" t="inlineStr">
+      <c r="X112" t="inlineStr">
         <is>
           <t>35527</t>
         </is>
@@ -6868,7 +6898,7 @@
           <t>HOLMER Erik</t>
         </is>
       </c>
-      <c r="U113" t="inlineStr">
+      <c r="X113" t="inlineStr">
         <is>
           <t>35104</t>
         </is>
@@ -6926,7 +6956,7 @@
           <t>SILVA Ivan</t>
         </is>
       </c>
-      <c r="U114" t="inlineStr">
+      <c r="X114" t="inlineStr">
         <is>
           <t>35482</t>
         </is>
@@ -6984,7 +7014,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U115" t="inlineStr">
+      <c r="X115" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -7042,7 +7072,7 @@
           <t>NABASKUES Unai</t>
         </is>
       </c>
-      <c r="U116" t="inlineStr">
+      <c r="X116" t="inlineStr">
         <is>
           <t>38775</t>
         </is>
@@ -7153,7 +7183,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U118" t="inlineStr">
+      <c r="X118" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -7211,7 +7241,7 @@
           <t>OSCHMAUTZ Felix</t>
         </is>
       </c>
-      <c r="U119" t="inlineStr">
+      <c r="X119" t="inlineStr">
         <is>
           <t>51856</t>
         </is>
@@ -7269,7 +7299,7 @@
           <t>POTOCNY Marcel</t>
         </is>
       </c>
-      <c r="U120" t="inlineStr">
+      <c r="X120" t="inlineStr">
         <is>
           <t>35235</t>
         </is>
@@ -7327,7 +7357,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U121" t="inlineStr">
+      <c r="X121" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -7385,7 +7415,7 @@
           <t>LEITNER Mario</t>
         </is>
       </c>
-      <c r="U122" t="inlineStr">
+      <c r="X122" t="inlineStr">
         <is>
           <t>35546</t>
         </is>
@@ -7443,7 +7473,7 @@
           <t>HUJSA Matus</t>
         </is>
       </c>
-      <c r="U123" t="inlineStr">
+      <c r="X123" t="inlineStr">
         <is>
           <t>35503</t>
         </is>
@@ -7501,7 +7531,7 @@
           <t>POWELL Richard</t>
         </is>
       </c>
-      <c r="U124" t="inlineStr">
+      <c r="X124" t="inlineStr">
         <is>
           <t>36444</t>
         </is>
@@ -7612,7 +7642,7 @@
           <t>FORBES-CRYANS Bradley</t>
         </is>
       </c>
-      <c r="U126" t="inlineStr">
+      <c r="X126" t="inlineStr">
         <is>
           <t>36513</t>
         </is>
@@ -7670,7 +7700,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U127" t="inlineStr">
+      <c r="X127" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -7728,7 +7758,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U128" t="inlineStr">
+      <c r="X128" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -7786,7 +7816,7 @@
           <t>BOECKELMANN Paul</t>
         </is>
       </c>
-      <c r="U129" t="inlineStr">
+      <c r="X129" t="inlineStr">
         <is>
           <t>35118</t>
         </is>
@@ -7844,7 +7874,7 @@
           <t>DAILLE Etienne</t>
         </is>
       </c>
-      <c r="U130" t="inlineStr">
+      <c r="X130" t="inlineStr">
         <is>
           <t>35308</t>
         </is>
@@ -7955,7 +7985,7 @@
           <t>MEGLIC Jure</t>
         </is>
       </c>
-      <c r="U132" t="inlineStr">
+      <c r="X132" t="inlineStr">
         <is>
           <t>35590</t>
         </is>
@@ -8013,7 +8043,7 @@
           <t>HAYWARD Ben</t>
         </is>
       </c>
-      <c r="U133" t="inlineStr">
+      <c r="X133" t="inlineStr">
         <is>
           <t>35539</t>
         </is>
@@ -8071,7 +8101,7 @@
           <t>BRUS Simon</t>
         </is>
       </c>
-      <c r="U134" t="inlineStr">
+      <c r="X134" t="inlineStr">
         <is>
           <t>39076</t>
         </is>
@@ -8129,7 +8159,7 @@
           <t>RENIA Benjamin</t>
         </is>
       </c>
-      <c r="U135" t="inlineStr">
+      <c r="X135" t="inlineStr">
         <is>
           <t>35407</t>
         </is>
@@ -8187,7 +8217,7 @@
           <t>HILGERT Lubos</t>
         </is>
       </c>
-      <c r="U136" t="inlineStr">
+      <c r="X136" t="inlineStr">
         <is>
           <t>35032</t>
         </is>
@@ -8245,7 +8275,7 @@
           <t>ALBREHT Martin</t>
         </is>
       </c>
-      <c r="U137" t="inlineStr">
+      <c r="X137" t="inlineStr">
         <is>
           <t>36898</t>
         </is>
@@ -8303,7 +8333,7 @@
           <t>PETERLIN Janos</t>
         </is>
       </c>
-      <c r="U138" t="inlineStr">
+      <c r="X138" t="inlineStr">
         <is>
           <t>36268</t>
         </is>
@@ -8361,7 +8391,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U139" t="inlineStr">
+      <c r="X139" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -8419,7 +8449,7 @@
           <t>CRESPO Joan</t>
         </is>
       </c>
-      <c r="U140" t="inlineStr">
+      <c r="X140" t="inlineStr">
         <is>
           <t>35749</t>
         </is>
@@ -8477,7 +8507,7 @@
           <t>ROMEO Andrea</t>
         </is>
       </c>
-      <c r="U141" t="inlineStr">
+      <c r="X141" t="inlineStr">
         <is>
           <t>35502</t>
         </is>
@@ -8535,7 +8565,7 @@
           <t>DOBY Mathieu</t>
         </is>
       </c>
-      <c r="U142" t="inlineStr">
+      <c r="X142" t="inlineStr">
         <is>
           <t>35292</t>
         </is>
@@ -8593,7 +8623,7 @@
           <t>HALCIN Martin</t>
         </is>
       </c>
-      <c r="U143" t="inlineStr">
+      <c r="X143" t="inlineStr">
         <is>
           <t>35355</t>
         </is>
@@ -8651,7 +8681,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U144" t="inlineStr">
+      <c r="X144" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -8709,7 +8739,7 @@
           <t>MOLMENTI Daniele</t>
         </is>
       </c>
-      <c r="U145" t="inlineStr">
+      <c r="X145" t="inlineStr">
         <is>
           <t>42017</t>
         </is>
@@ -8767,7 +8797,7 @@
           <t>BERSINGER Thomas</t>
         </is>
       </c>
-      <c r="U146" t="inlineStr">
+      <c r="X146" t="inlineStr">
         <is>
           <t>35228</t>
         </is>
@@ -8825,7 +8855,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U147" t="inlineStr">
+      <c r="X147" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -8883,7 +8913,7 @@
           <t>GRIMM Alexander</t>
         </is>
       </c>
-      <c r="U148" t="inlineStr">
+      <c r="X148" t="inlineStr">
         <is>
           <t>35112</t>
         </is>
@@ -8941,7 +8971,7 @@
           <t>TUNKA Ondrej</t>
         </is>
       </c>
-      <c r="U149" t="inlineStr">
+      <c r="X149" t="inlineStr">
         <is>
           <t>35947</t>
         </is>
@@ -8999,7 +9029,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U150" t="inlineStr">
+      <c r="X150" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -9057,7 +9087,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U151" t="inlineStr">
+      <c r="X151" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -9115,7 +9145,7 @@
           <t>BIAZIZZO Mathieu</t>
         </is>
       </c>
-      <c r="U152" t="inlineStr">
+      <c r="X152" t="inlineStr">
         <is>
           <t>35484</t>
         </is>
@@ -9173,7 +9203,7 @@
           <t>SCHUBERT Sebastian</t>
         </is>
       </c>
-      <c r="U153" t="inlineStr">
+      <c r="X153" t="inlineStr">
         <is>
           <t>35114</t>
         </is>
@@ -9231,7 +9261,7 @@
           <t>ROSSI Lucas</t>
         </is>
       </c>
-      <c r="U154" t="inlineStr">
+      <c r="X154" t="inlineStr">
         <is>
           <t>36925</t>
         </is>
@@ -9289,7 +9319,7 @@
           <t>MARZO Daniel</t>
         </is>
       </c>
-      <c r="U155" t="inlineStr">
+      <c r="X155" t="inlineStr">
         <is>
           <t>35757</t>
         </is>
@@ -9347,7 +9377,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U156" t="inlineStr">
+      <c r="X156" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -9405,7 +9435,7 @@
           <t>DOBY Mathieu</t>
         </is>
       </c>
-      <c r="U157" t="inlineStr">
+      <c r="X157" t="inlineStr">
         <is>
           <t>35292</t>
         </is>
@@ -9463,7 +9493,7 @@
           <t>LONG Tren</t>
         </is>
       </c>
-      <c r="U158" t="inlineStr">
+      <c r="X158" t="inlineStr">
         <is>
           <t>57124</t>
         </is>
@@ -9521,7 +9551,7 @@
           <t>SMITH Tyler</t>
         </is>
       </c>
-      <c r="U159" t="inlineStr">
+      <c r="X159" t="inlineStr">
         <is>
           <t>51904</t>
         </is>
@@ -9579,7 +9609,7 @@
           <t>JEKLIN Jakob</t>
         </is>
       </c>
-      <c r="U160" t="inlineStr">
+      <c r="X160" t="inlineStr">
         <is>
           <t>42022</t>
         </is>
@@ -9637,7 +9667,7 @@
           <t>SOSA Angelo</t>
         </is>
       </c>
-      <c r="U161" t="inlineStr">
+      <c r="X161" t="inlineStr">
         <is>
           <t>51793</t>
         </is>
@@ -9695,7 +9725,7 @@
           <t>WASHER Patrick</t>
         </is>
       </c>
-      <c r="U162" t="inlineStr">
+      <c r="X162" t="inlineStr">
         <is>
           <t>42081</t>
         </is>
@@ -9753,7 +9783,7 @@
           <t>SILVA Jose</t>
         </is>
       </c>
-      <c r="U163" t="inlineStr">
+      <c r="X163" t="inlineStr">
         <is>
           <t>36494</t>
         </is>
@@ -9811,7 +9841,7 @@
           <t>CORREA Charles</t>
         </is>
       </c>
-      <c r="U164" t="inlineStr">
+      <c r="X164" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
@@ -9869,7 +9899,7 @@
           <t>PARES Lluis</t>
         </is>
       </c>
-      <c r="U165" t="inlineStr">
+      <c r="X165" t="inlineStr">
         <is>
           <t>44008</t>
         </is>
@@ -9927,7 +9957,7 @@
           <t>GIBB Benjamin</t>
         </is>
       </c>
-      <c r="U166" t="inlineStr">
+      <c r="X166" t="inlineStr">
         <is>
           <t>36711</t>
         </is>
@@ -9985,7 +10015,7 @@
           <t>CHEN Fangjia</t>
         </is>
       </c>
-      <c r="U167" t="inlineStr">
+      <c r="X167" t="inlineStr">
         <is>
           <t>42638</t>
         </is>
@@ -10043,7 +10073,7 @@
           <t>CURCEL Leonardo</t>
         </is>
       </c>
-      <c r="U168" t="inlineStr">
+      <c r="X168" t="inlineStr">
         <is>
           <t>38014</t>
         </is>
@@ -10101,7 +10131,7 @@
           <t>GARMENDIA Aitor</t>
         </is>
       </c>
-      <c r="U169" t="inlineStr">
+      <c r="X169" t="inlineStr">
         <is>
           <t>35745</t>
         </is>
@@ -10212,7 +10242,7 @@
           <t>CECCON Paolo</t>
         </is>
       </c>
-      <c r="U171" t="inlineStr">
+      <c r="X171" t="inlineStr">
         <is>
           <t>39903</t>
         </is>
@@ -10270,7 +10300,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U172" t="inlineStr">
+      <c r="X172" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -10328,7 +10358,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U173" t="inlineStr">
+      <c r="X173" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -10386,7 +10416,7 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U174" t="inlineStr">
+      <c r="X174" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -10550,7 +10580,7 @@
           <t>CIPRESSI Stefano</t>
         </is>
       </c>
-      <c r="U177" t="inlineStr">
+      <c r="X177" t="inlineStr">
         <is>
           <t>35495</t>
         </is>
@@ -10608,7 +10638,7 @@
           <t>NAVEAU Laurine</t>
         </is>
       </c>
-      <c r="U178" t="inlineStr">
+      <c r="X178" t="inlineStr">
         <is>
           <t>53246</t>
         </is>
@@ -10666,7 +10696,7 @@
           <t>GLEJTEKOVA Simona</t>
         </is>
       </c>
-      <c r="U179" t="inlineStr">
+      <c r="X179" t="inlineStr">
         <is>
           <t>55166</t>
         </is>
@@ -10724,7 +10754,7 @@
           <t>SKACHOVA Monika</t>
         </is>
       </c>
-      <c r="U180" t="inlineStr">
+      <c r="X180" t="inlineStr">
         <is>
           <t>53078</t>
         </is>
@@ -10782,7 +10812,7 @@
           <t>MACEKOVA Simona</t>
         </is>
       </c>
-      <c r="U181" t="inlineStr">
+      <c r="X181" t="inlineStr">
         <is>
           <t>45153</t>
         </is>
@@ -10893,7 +10923,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U183" t="inlineStr">
+      <c r="X183" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -10951,7 +10981,7 @@
           <t>DANIELS Haley</t>
         </is>
       </c>
-      <c r="U184" t="inlineStr">
+      <c r="X184" t="inlineStr">
         <is>
           <t>36260</t>
         </is>
@@ -11009,7 +11039,7 @@
           <t>RANKIN Georgia</t>
         </is>
       </c>
-      <c r="U185" t="inlineStr">
+      <c r="X185" t="inlineStr">
         <is>
           <t>38435</t>
         </is>
@@ -11067,7 +11097,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U186" t="inlineStr">
+      <c r="X186" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -11125,7 +11155,7 @@
           <t>BORROWS Alison</t>
         </is>
       </c>
-      <c r="U187" t="inlineStr">
+      <c r="X187" t="inlineStr">
         <is>
           <t>38440</t>
         </is>
@@ -11183,7 +11213,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U188" t="inlineStr">
+      <c r="X188" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -11241,7 +11271,7 @@
           <t>SOARES Renan</t>
         </is>
       </c>
-      <c r="U189" t="inlineStr">
+      <c r="X189" t="inlineStr">
         <is>
           <t>42776</t>
         </is>
@@ -11352,7 +11382,7 @@
           <t>AKINYEMI Johnathan</t>
         </is>
       </c>
-      <c r="U191" t="inlineStr">
+      <c r="X191" t="inlineStr">
         <is>
           <t>36822</t>
         </is>
@@ -11463,7 +11493,7 @@
           <t>SWETNAM Huw</t>
         </is>
       </c>
-      <c r="U193" t="inlineStr">
+      <c r="X193" t="inlineStr">
         <is>
           <t>35652</t>
         </is>
@@ -11521,7 +11551,7 @@
           <t>WESTFALL Tyler</t>
         </is>
       </c>
-      <c r="U194" t="inlineStr">
+      <c r="X194" t="inlineStr">
         <is>
           <t>51919</t>
         </is>
@@ -11579,7 +11609,7 @@
           <t>MAPELLI Guilherme Marcello</t>
         </is>
       </c>
-      <c r="U195" t="inlineStr">
+      <c r="X195" t="inlineStr">
         <is>
           <t>38015</t>
         </is>
@@ -11637,7 +11667,7 @@
           <t>OGURA Takashi</t>
         </is>
       </c>
-      <c r="U196" t="inlineStr">
+      <c r="X196" t="inlineStr">
         <is>
           <t>37679</t>
         </is>
@@ -11695,7 +11725,7 @@
           <t>STANOVSKY Martin</t>
         </is>
       </c>
-      <c r="U197" t="inlineStr">
+      <c r="X197" t="inlineStr">
         <is>
           <t>68782</t>
         </is>
@@ -11753,7 +11783,7 @@
           <t>WEGER Jakob</t>
         </is>
       </c>
-      <c r="U198" t="inlineStr">
+      <c r="X198" t="inlineStr">
         <is>
           <t>54909</t>
         </is>
@@ -11811,7 +11841,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U199" t="inlineStr">
+      <c r="X199" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -11869,7 +11899,7 @@
           <t>SMITH Tyler</t>
         </is>
       </c>
-      <c r="U200" t="inlineStr">
+      <c r="X200" t="inlineStr">
         <is>
           <t>51904</t>
         </is>
@@ -11927,7 +11957,7 @@
           <t>QUAN Xin</t>
         </is>
       </c>
-      <c r="U201" t="inlineStr">
+      <c r="X201" t="inlineStr">
         <is>
           <t>62343</t>
         </is>
@@ -11985,7 +12015,7 @@
           <t>CORTEZ Geronimo</t>
         </is>
       </c>
-      <c r="U202" t="inlineStr">
+      <c r="X202" t="inlineStr">
         <is>
           <t>51835</t>
         </is>
@@ -12043,7 +12073,7 @@
           <t>PEREZ Alexis</t>
         </is>
       </c>
-      <c r="U203" t="inlineStr">
+      <c r="X203" t="inlineStr">
         <is>
           <t>41649</t>
         </is>
@@ -12101,7 +12131,7 @@
           <t>ROSSI Lucas</t>
         </is>
       </c>
-      <c r="U204" t="inlineStr">
+      <c r="X204" t="inlineStr">
         <is>
           <t>36925</t>
         </is>
@@ -12159,7 +12189,7 @@
           <t>MARTINS TAQUES Ricardo</t>
         </is>
       </c>
-      <c r="U205" t="inlineStr">
+      <c r="X205" t="inlineStr">
         <is>
           <t>38022</t>
         </is>
@@ -12217,7 +12247,7 @@
           <t>MARTIN Gerome</t>
         </is>
       </c>
-      <c r="U206" t="inlineStr">
+      <c r="X206" t="inlineStr">
         <is>
           <t>36720</t>
         </is>
@@ -12275,7 +12305,7 @@
           <t>WEGER Matthias</t>
         </is>
       </c>
-      <c r="U207" t="inlineStr">
+      <c r="X207" t="inlineStr">
         <is>
           <t>68837</t>
         </is>
@@ -12333,7 +12363,7 @@
           <t>WAHLEN Fredrik</t>
         </is>
       </c>
-      <c r="U208" t="inlineStr">
+      <c r="X208" t="inlineStr">
         <is>
           <t>35102</t>
         </is>
@@ -12391,7 +12421,7 @@
           <t>TAN Ya</t>
         </is>
       </c>
-      <c r="U209" t="inlineStr">
+      <c r="X209" t="inlineStr">
         <is>
           <t>52024</t>
         </is>
@@ -12449,7 +12479,7 @@
           <t>SCHLAEFLI Jeremias</t>
         </is>
       </c>
-      <c r="U210" t="inlineStr">
+      <c r="X210" t="inlineStr">
         <is>
           <t>35430</t>
         </is>
@@ -12507,7 +12537,7 @@
           <t>TSVIET Igor</t>
         </is>
       </c>
-      <c r="U211" t="inlineStr">
+      <c r="X211" t="inlineStr">
         <is>
           <t>35527</t>
         </is>
@@ -12565,7 +12595,7 @@
           <t>HOLMER Erik</t>
         </is>
       </c>
-      <c r="U212" t="inlineStr">
+      <c r="X212" t="inlineStr">
         <is>
           <t>35104</t>
         </is>
@@ -12623,7 +12653,7 @@
           <t>SILVA Ivan</t>
         </is>
       </c>
-      <c r="U213" t="inlineStr">
+      <c r="X213" t="inlineStr">
         <is>
           <t>35482</t>
         </is>
@@ -12681,7 +12711,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U214" t="inlineStr">
+      <c r="X214" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -12739,7 +12769,7 @@
           <t>NABASKUES Unai</t>
         </is>
       </c>
-      <c r="U215" t="inlineStr">
+      <c r="X215" t="inlineStr">
         <is>
           <t>38775</t>
         </is>
@@ -12797,7 +12827,7 @@
           <t>OSCHMAUTZ Felix</t>
         </is>
       </c>
-      <c r="U216" t="inlineStr">
+      <c r="X216" t="inlineStr">
         <is>
           <t>51856</t>
         </is>
@@ -12855,7 +12885,7 @@
           <t>POTOCNY Marcel</t>
         </is>
       </c>
-      <c r="U217" t="inlineStr">
+      <c r="X217" t="inlineStr">
         <is>
           <t>35235</t>
         </is>
@@ -12913,7 +12943,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U218" t="inlineStr">
+      <c r="X218" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -13024,7 +13054,7 @@
           <t>MALEK Andrej</t>
         </is>
       </c>
-      <c r="U220" t="inlineStr">
+      <c r="X220" t="inlineStr">
         <is>
           <t>39246</t>
         </is>
@@ -13082,7 +13112,7 @@
           <t>DAILLE Etienne</t>
         </is>
       </c>
-      <c r="U221" t="inlineStr">
+      <c r="X221" t="inlineStr">
         <is>
           <t>35308</t>
         </is>
@@ -13193,7 +13223,7 @@
           <t>HAYWARD Ben</t>
         </is>
       </c>
-      <c r="U223" t="inlineStr">
+      <c r="X223" t="inlineStr">
         <is>
           <t>35539</t>
         </is>
@@ -13251,7 +13281,7 @@
           <t>BRUS Simon</t>
         </is>
       </c>
-      <c r="U224" t="inlineStr">
+      <c r="X224" t="inlineStr">
         <is>
           <t>39076</t>
         </is>
@@ -13309,7 +13339,7 @@
           <t>HILGERT Lubos</t>
         </is>
       </c>
-      <c r="U225" t="inlineStr">
+      <c r="X225" t="inlineStr">
         <is>
           <t>35032</t>
         </is>
@@ -13367,7 +13397,7 @@
           <t>PETERLIN Janos</t>
         </is>
       </c>
-      <c r="U226" t="inlineStr">
+      <c r="X226" t="inlineStr">
         <is>
           <t>36268</t>
         </is>
@@ -13425,7 +13455,7 @@
           <t>ROMEO Andrea</t>
         </is>
       </c>
-      <c r="U227" t="inlineStr">
+      <c r="X227" t="inlineStr">
         <is>
           <t>35502</t>
         </is>
@@ -13589,7 +13619,7 @@
           <t>GRAILLE Solene</t>
         </is>
       </c>
-      <c r="U230" t="inlineStr">
+      <c r="X230" t="inlineStr">
         <is>
           <t>36211</t>
         </is>
@@ -13647,7 +13677,7 @@
           <t>CASSINI Maria Luz</t>
         </is>
       </c>
-      <c r="U231" t="inlineStr">
+      <c r="X231" t="inlineStr">
         <is>
           <t>41627</t>
         </is>
@@ -13705,7 +13735,7 @@
           <t>HIGGINS Anna</t>
         </is>
       </c>
-      <c r="U232" t="inlineStr">
+      <c r="X232" t="inlineStr">
         <is>
           <t>42107</t>
         </is>
@@ -13816,7 +13846,7 @@
           <t>IFARRAGUERRI Anna Maria</t>
         </is>
       </c>
-      <c r="U234" t="inlineStr">
+      <c r="X234" t="inlineStr">
         <is>
           <t>39209</t>
         </is>
@@ -13874,7 +13904,7 @@
           <t>EGUES Irene</t>
         </is>
       </c>
-      <c r="U235" t="inlineStr">
+      <c r="X235" t="inlineStr">
         <is>
           <t>51854</t>
         </is>
@@ -13932,7 +13962,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U236" t="inlineStr">
+      <c r="X236" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -14043,7 +14073,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U238" t="inlineStr">
+      <c r="X238" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -14101,7 +14131,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U239" t="inlineStr">
+      <c r="X239" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -14159,7 +14189,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U240" t="inlineStr">
+      <c r="X240" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -14217,7 +14247,7 @@
           <t>GROENEVELD Jessica</t>
         </is>
       </c>
-      <c r="U241" t="inlineStr">
+      <c r="X241" t="inlineStr">
         <is>
           <t>35542</t>
         </is>
@@ -14328,7 +14358,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U243" t="inlineStr">
+      <c r="X243" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -14386,7 +14416,7 @@
           <t>SABATTINI Chiara</t>
         </is>
       </c>
-      <c r="U244" t="inlineStr">
+      <c r="X244" t="inlineStr">
         <is>
           <t>35219</t>
         </is>
@@ -14444,7 +14474,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U245" t="inlineStr">
+      <c r="X245" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -14502,7 +14532,7 @@
           <t>GUIET Pauline</t>
         </is>
       </c>
-      <c r="U246" t="inlineStr">
+      <c r="X246" t="inlineStr">
         <is>
           <t>35493</t>
         </is>
@@ -14560,7 +14590,7 @@
           <t>LI Tong</t>
         </is>
       </c>
-      <c r="U247" t="inlineStr">
+      <c r="X247" t="inlineStr">
         <is>
           <t>52023</t>
         </is>
@@ -14618,7 +14648,7 @@
           <t>GIAI PRON Maria Clara</t>
         </is>
       </c>
-      <c r="U248" t="inlineStr">
+      <c r="X248" t="inlineStr">
         <is>
           <t>35218</t>
         </is>
@@ -14676,7 +14706,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U249" t="inlineStr">
+      <c r="X249" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -14734,7 +14764,7 @@
           <t>NEVARILOVA Kristina</t>
         </is>
       </c>
-      <c r="U250" t="inlineStr">
+      <c r="X250" t="inlineStr">
         <is>
           <t>35467</t>
         </is>
@@ -14792,7 +14822,7 @@
           <t>MANGIN Estelle</t>
         </is>
       </c>
-      <c r="U251" t="inlineStr">
+      <c r="X251" t="inlineStr">
         <is>
           <t>35670</t>
         </is>
@@ -14850,7 +14880,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U252" t="inlineStr">
+      <c r="X252" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -14908,7 +14938,7 @@
           <t>GOIKOETXEA Irati</t>
         </is>
       </c>
-      <c r="U253" t="inlineStr">
+      <c r="X253" t="inlineStr">
         <is>
           <t>35761</t>
         </is>
@@ -14966,7 +14996,7 @@
           <t>BOUZIDI Carole</t>
         </is>
       </c>
-      <c r="U254" t="inlineStr">
+      <c r="X254" t="inlineStr">
         <is>
           <t>35231</t>
         </is>
@@ -15024,7 +15054,7 @@
           <t>OBLINGER-PETERS Violetta</t>
         </is>
       </c>
-      <c r="U255" t="inlineStr">
+      <c r="X255" t="inlineStr">
         <is>
           <t>35289</t>
         </is>
@@ -15082,7 +15112,7 @@
           <t>KALISKA Elena</t>
         </is>
       </c>
-      <c r="U256" t="inlineStr">
+      <c r="X256" t="inlineStr">
         <is>
           <t>35366</t>
         </is>
@@ -15140,7 +15170,7 @@
           <t>LI Lu</t>
         </is>
       </c>
-      <c r="U257" t="inlineStr">
+      <c r="X257" t="inlineStr">
         <is>
           <t>37086</t>
         </is>
@@ -15198,7 +15228,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U258" t="inlineStr">
+      <c r="X258" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -15256,7 +15286,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U259" t="inlineStr">
+      <c r="X259" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -15367,7 +15397,7 @@
           <t>LEITNER Lisa</t>
         </is>
       </c>
-      <c r="U261" t="inlineStr">
+      <c r="X261" t="inlineStr">
         <is>
           <t>35305</t>
         </is>
@@ -15425,7 +15455,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U262" t="inlineStr">
+      <c r="X262" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -15483,7 +15513,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U263" t="inlineStr">
+      <c r="X263" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -15541,7 +15571,7 @@
           <t>MARTINEZ Marta</t>
         </is>
       </c>
-      <c r="U264" t="inlineStr">
+      <c r="X264" t="inlineStr">
         <is>
           <t>35760</t>
         </is>
@@ -15599,7 +15629,7 @@
           <t>HILGERTOVA Stepanka</t>
         </is>
       </c>
-      <c r="U265" t="inlineStr">
+      <c r="X265" t="inlineStr">
         <is>
           <t>35035</t>
         </is>
@@ -15657,7 +15687,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U266" t="inlineStr">
+      <c r="X266" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -15715,7 +15745,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U267" t="inlineStr">
+      <c r="X267" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -15773,7 +15803,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U268" t="inlineStr">
+      <c r="X268" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -15831,7 +15861,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U269" t="inlineStr">
+      <c r="X269" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -15889,7 +15919,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U270" t="inlineStr">
+      <c r="X270" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -15952,12 +15982,12 @@
           <t>VIEIRA Cassiano</t>
         </is>
       </c>
-      <c r="U271" t="inlineStr">
+      <c r="X271" t="inlineStr">
         <is>
           <t>42977</t>
         </is>
       </c>
-      <c r="V271" t="inlineStr">
+      <c r="Y271" t="inlineStr">
         <is>
           <t>42976</t>
         </is>
@@ -16020,12 +16050,12 @@
           <t>KASPAR Albert</t>
         </is>
       </c>
-      <c r="U272" t="inlineStr">
+      <c r="X272" t="inlineStr">
         <is>
           <t>42012</t>
         </is>
       </c>
-      <c r="V272" t="inlineStr">
+      <c r="Y272" t="inlineStr">
         <is>
           <t>42013</t>
         </is>
@@ -16088,12 +16118,12 @@
           <t>CHEN Jin</t>
         </is>
       </c>
-      <c r="U273" t="inlineStr">
+      <c r="X273" t="inlineStr">
         <is>
           <t>42237</t>
         </is>
       </c>
-      <c r="V273" t="inlineStr">
+      <c r="Y273" t="inlineStr">
         <is>
           <t>42238</t>
         </is>
@@ -16156,12 +16186,12 @@
           <t>DENG Xiao</t>
         </is>
       </c>
-      <c r="U274" t="inlineStr">
+      <c r="X274" t="inlineStr">
         <is>
           <t>42239</t>
         </is>
       </c>
-      <c r="V274" t="inlineStr">
+      <c r="Y274" t="inlineStr">
         <is>
           <t>42240</t>
         </is>
@@ -16224,12 +16254,12 @@
           <t>OLIVEIRA Anderson</t>
         </is>
       </c>
-      <c r="U275" t="inlineStr">
+      <c r="X275" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
       </c>
-      <c r="V275" t="inlineStr">
+      <c r="Y275" t="inlineStr">
         <is>
           <t>38020</t>
         </is>
@@ -16292,12 +16322,12 @@
           <t>LE RUYET Edern</t>
         </is>
       </c>
-      <c r="U276" t="inlineStr">
+      <c r="X276" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
       </c>
-      <c r="V276" t="inlineStr">
+      <c r="Y276" t="inlineStr">
         <is>
           <t>35379</t>
         </is>
@@ -16360,12 +16390,12 @@
           <t>CAILHOL Hugo</t>
         </is>
       </c>
-      <c r="U277" t="inlineStr">
+      <c r="X277" t="inlineStr">
         <is>
           <t>35476</t>
         </is>
       </c>
-      <c r="V277" t="inlineStr">
+      <c r="Y277" t="inlineStr">
         <is>
           <t>35491</t>
         </is>
@@ -16428,12 +16458,12 @@
           <t>KERVELLA Loic</t>
         </is>
       </c>
-      <c r="U278" t="inlineStr">
+      <c r="X278" t="inlineStr">
         <is>
           <t>35671</t>
         </is>
       </c>
-      <c r="V278" t="inlineStr">
+      <c r="Y278" t="inlineStr">
         <is>
           <t>35672</t>
         </is>
@@ -16496,12 +16526,12 @@
           <t>FERRARI Niccolo</t>
         </is>
       </c>
-      <c r="U279" t="inlineStr">
+      <c r="X279" t="inlineStr">
         <is>
           <t>35497</t>
         </is>
       </c>
-      <c r="V279" t="inlineStr">
+      <c r="Y279" t="inlineStr">
         <is>
           <t>35498</t>
         </is>
@@ -16564,12 +16594,12 @@
           <t>HOCHSCHORNER Peter</t>
         </is>
       </c>
-      <c r="U280" t="inlineStr">
+      <c r="X280" t="inlineStr">
         <is>
           <t>35356</t>
         </is>
       </c>
-      <c r="V280" t="inlineStr">
+      <c r="Y280" t="inlineStr">
         <is>
           <t>35357</t>
         </is>
@@ -16632,12 +16662,12 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U281" t="inlineStr">
+      <c r="X281" t="inlineStr">
         <is>
           <t>35145</t>
         </is>
       </c>
-      <c r="V281" t="inlineStr">
+      <c r="Y281" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -16700,12 +16730,12 @@
           <t>PEREZ Jesus</t>
         </is>
       </c>
-      <c r="U282" t="inlineStr">
+      <c r="X282" t="inlineStr">
         <is>
           <t>35757</t>
         </is>
       </c>
-      <c r="V282" t="inlineStr">
+      <c r="Y282" t="inlineStr">
         <is>
           <t>36091</t>
         </is>
@@ -16768,12 +16798,12 @@
           <t>MUELLER Kevin</t>
         </is>
       </c>
-      <c r="U283" t="inlineStr">
+      <c r="X283" t="inlineStr">
         <is>
           <t>35148</t>
         </is>
       </c>
-      <c r="V283" t="inlineStr">
+      <c r="Y283" t="inlineStr">
         <is>
           <t>35149</t>
         </is>
@@ -16836,12 +16866,12 @@
           <t>BATIK Jan</t>
         </is>
       </c>
-      <c r="U284" t="inlineStr">
+      <c r="X284" t="inlineStr">
         <is>
           <t>35368</t>
         </is>
       </c>
-      <c r="V284" t="inlineStr">
+      <c r="Y284" t="inlineStr">
         <is>
           <t>35367</t>
         </is>
@@ -16904,12 +16934,12 @@
           <t>BECKER Thomas</t>
         </is>
       </c>
-      <c r="U285" t="inlineStr">
+      <c r="X285" t="inlineStr">
         <is>
           <t>35139</t>
         </is>
       </c>
-      <c r="V285" t="inlineStr">
+      <c r="Y285" t="inlineStr">
         <is>
           <t>35143</t>
         </is>
@@ -16972,12 +17002,12 @@
           <t>JANE Jakub</t>
         </is>
       </c>
-      <c r="U286" t="inlineStr">
+      <c r="X286" t="inlineStr">
         <is>
           <t>35060</t>
         </is>
       </c>
-      <c r="V286" t="inlineStr">
+      <c r="Y286" t="inlineStr">
         <is>
           <t>35061</t>
         </is>
@@ -17040,12 +17070,12 @@
           <t>BISO Hugo</t>
         </is>
       </c>
-      <c r="U287" t="inlineStr">
+      <c r="X287" t="inlineStr">
         <is>
           <t>35403</t>
         </is>
       </c>
-      <c r="V287" t="inlineStr">
+      <c r="Y287" t="inlineStr">
         <is>
           <t>35229</t>
         </is>
@@ -17103,7 +17133,7 @@
           <t>GRAILLE Solene</t>
         </is>
       </c>
-      <c r="U288" t="inlineStr">
+      <c r="X288" t="inlineStr">
         <is>
           <t>36211</t>
         </is>
@@ -17161,7 +17191,7 @@
           <t>CASSINI Maria Luz</t>
         </is>
       </c>
-      <c r="U289" t="inlineStr">
+      <c r="X289" t="inlineStr">
         <is>
           <t>41627</t>
         </is>
@@ -17219,7 +17249,7 @@
           <t>HIGGINS Anna</t>
         </is>
       </c>
-      <c r="U290" t="inlineStr">
+      <c r="X290" t="inlineStr">
         <is>
           <t>42107</t>
         </is>
@@ -17330,7 +17360,7 @@
           <t>IFARRAGUERRI Anna Maria</t>
         </is>
       </c>
-      <c r="U292" t="inlineStr">
+      <c r="X292" t="inlineStr">
         <is>
           <t>39209</t>
         </is>
@@ -17388,7 +17418,7 @@
           <t>EGUES Irene</t>
         </is>
       </c>
-      <c r="U293" t="inlineStr">
+      <c r="X293" t="inlineStr">
         <is>
           <t>51854</t>
         </is>
@@ -17446,7 +17476,7 @@
           <t>ECKHARDT Kate</t>
         </is>
       </c>
-      <c r="U294" t="inlineStr">
+      <c r="X294" t="inlineStr">
         <is>
           <t>44815</t>
         </is>
@@ -17557,7 +17587,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U296" t="inlineStr">
+      <c r="X296" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -17615,7 +17645,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U297" t="inlineStr">
+      <c r="X297" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -17673,7 +17703,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U298" t="inlineStr">
+      <c r="X298" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -17731,7 +17761,7 @@
           <t>GROENEVELD Jessica</t>
         </is>
       </c>
-      <c r="U299" t="inlineStr">
+      <c r="X299" t="inlineStr">
         <is>
           <t>35542</t>
         </is>
@@ -17842,7 +17872,7 @@
           <t>SABATTINI Chiara</t>
         </is>
       </c>
-      <c r="U301" t="inlineStr">
+      <c r="X301" t="inlineStr">
         <is>
           <t>35219</t>
         </is>
@@ -17900,7 +17930,7 @@
           <t>NOVAK Ajda</t>
         </is>
       </c>
-      <c r="U302" t="inlineStr">
+      <c r="X302" t="inlineStr">
         <is>
           <t>39079</t>
         </is>
@@ -17958,7 +17988,7 @@
           <t>LI Tong</t>
         </is>
       </c>
-      <c r="U303" t="inlineStr">
+      <c r="X303" t="inlineStr">
         <is>
           <t>52023</t>
         </is>
@@ -18016,7 +18046,7 @@
           <t>GIAI PRON Maria Clara</t>
         </is>
       </c>
-      <c r="U304" t="inlineStr">
+      <c r="X304" t="inlineStr">
         <is>
           <t>35218</t>
         </is>
@@ -18074,7 +18104,7 @@
           <t>NEVARILOVA Kristina</t>
         </is>
       </c>
-      <c r="U305" t="inlineStr">
+      <c r="X305" t="inlineStr">
         <is>
           <t>35467</t>
         </is>
@@ -18132,7 +18162,7 @@
           <t>KALISKA Elena</t>
         </is>
       </c>
-      <c r="U306" t="inlineStr">
+      <c r="X306" t="inlineStr">
         <is>
           <t>35366</t>
         </is>
@@ -18243,7 +18273,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U308" t="inlineStr">
+      <c r="X308" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -18513,7 +18543,7 @@
           <t>MACEKOVA Simona</t>
         </is>
       </c>
-      <c r="U313" t="inlineStr">
+      <c r="X313" t="inlineStr">
         <is>
           <t>45153</t>
         </is>
@@ -18624,7 +18654,7 @@
           <t>GARMENDIA Aitor</t>
         </is>
       </c>
-      <c r="U315" t="inlineStr">
+      <c r="X315" t="inlineStr">
         <is>
           <t>35745</t>
         </is>
@@ -18682,7 +18712,7 @@
           <t>CORREA Charles</t>
         </is>
       </c>
-      <c r="U316" t="inlineStr">
+      <c r="X316" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
@@ -18740,7 +18770,7 @@
           <t>CURCEL Leonardo</t>
         </is>
       </c>
-      <c r="U317" t="inlineStr">
+      <c r="X317" t="inlineStr">
         <is>
           <t>38014</t>
         </is>
@@ -18798,7 +18828,7 @@
           <t>CHEN Fangjia</t>
         </is>
       </c>
-      <c r="U318" t="inlineStr">
+      <c r="X318" t="inlineStr">
         <is>
           <t>42638</t>
         </is>
@@ -18856,7 +18886,7 @@
           <t>CIPRESSI Stefano</t>
         </is>
       </c>
-      <c r="U319" t="inlineStr">
+      <c r="X319" t="inlineStr">
         <is>
           <t>35495</t>
         </is>
@@ -18914,7 +18944,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U320" t="inlineStr">
+      <c r="X320" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -19025,7 +19055,7 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U322" t="inlineStr">
+      <c r="X322" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -19136,7 +19166,7 @@
           <t>ROHAN Lukas</t>
         </is>
       </c>
-      <c r="U324" t="inlineStr">
+      <c r="X324" t="inlineStr">
         <is>
           <t>36114</t>
         </is>
@@ -19194,7 +19224,7 @@
           <t>LOKKEN Zachary</t>
         </is>
       </c>
-      <c r="U325" t="inlineStr">
+      <c r="X325" t="inlineStr">
         <is>
           <t>35069</t>
         </is>
@@ -19252,7 +19282,7 @@
           <t>FOULON Kilian</t>
         </is>
       </c>
-      <c r="U326" t="inlineStr">
+      <c r="X326" t="inlineStr">
         <is>
           <t>35602</t>
         </is>
@@ -19310,7 +19340,7 @@
           <t>SHU Jianming</t>
         </is>
       </c>
-      <c r="U327" t="inlineStr">
+      <c r="X327" t="inlineStr">
         <is>
           <t>47327</t>
         </is>
@@ -19368,7 +19398,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U328" t="inlineStr">
+      <c r="X328" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -19426,7 +19456,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U329" t="inlineStr">
+      <c r="X329" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -19484,7 +19514,7 @@
           <t>BORROWS Ian</t>
         </is>
       </c>
-      <c r="U330" t="inlineStr">
+      <c r="X330" t="inlineStr">
         <is>
           <t>36534</t>
         </is>
@@ -19542,7 +19572,7 @@
           <t>PESCHIER Nicolas</t>
         </is>
       </c>
-      <c r="U331" t="inlineStr">
+      <c r="X331" t="inlineStr">
         <is>
           <t>35401</t>
         </is>
@@ -19600,7 +19630,7 @@
           <t>COF Blaz</t>
         </is>
       </c>
-      <c r="U332" t="inlineStr">
+      <c r="X332" t="inlineStr">
         <is>
           <t>36897</t>
         </is>
@@ -19658,7 +19688,7 @@
           <t>JEGOU Liam</t>
         </is>
       </c>
-      <c r="U333" t="inlineStr">
+      <c r="X333" t="inlineStr">
         <is>
           <t>35820</t>
         </is>
@@ -19716,7 +19746,7 @@
           <t>THOMAS Martin</t>
         </is>
       </c>
-      <c r="U334" t="inlineStr">
+      <c r="X334" t="inlineStr">
         <is>
           <t>35412</t>
         </is>
@@ -19774,7 +19804,7 @@
           <t>BURGESS Adam</t>
         </is>
       </c>
-      <c r="U335" t="inlineStr">
+      <c r="X335" t="inlineStr">
         <is>
           <t>35647</t>
         </is>
@@ -19832,7 +19862,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U336" t="inlineStr">
+      <c r="X336" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -19890,7 +19920,7 @@
           <t>TILLARD Pierre-Antoine</t>
         </is>
       </c>
-      <c r="U337" t="inlineStr">
+      <c r="X337" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
@@ -19948,7 +19978,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U338" t="inlineStr">
+      <c r="X338" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -20006,7 +20036,7 @@
           <t>WESTLEY Ryan</t>
         </is>
       </c>
-      <c r="U339" t="inlineStr">
+      <c r="X339" t="inlineStr">
         <is>
           <t>35651</t>
         </is>
@@ -20064,7 +20094,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U340" t="inlineStr">
+      <c r="X340" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -20122,7 +20152,7 @@
           <t>SMEDLEY Cameron</t>
         </is>
       </c>
-      <c r="U341" t="inlineStr">
+      <c r="X341" t="inlineStr">
         <is>
           <t>35543</t>
         </is>
@@ -20180,7 +20210,7 @@
           <t>JANE Michal</t>
         </is>
       </c>
-      <c r="U342" t="inlineStr">
+      <c r="X342" t="inlineStr">
         <is>
           <t>35059</t>
         </is>
@@ -20238,7 +20268,7 @@
           <t>MIRGORODSKY Marko</t>
         </is>
       </c>
-      <c r="U343" t="inlineStr">
+      <c r="X343" t="inlineStr">
         <is>
           <t>42019</t>
         </is>
@@ -20296,7 +20326,7 @@
           <t>SLAFKOVSKY Alexander</t>
         </is>
       </c>
-      <c r="U344" t="inlineStr">
+      <c r="X344" t="inlineStr">
         <is>
           <t>35129</t>
         </is>
@@ -20354,7 +20384,7 @@
           <t>BORROWS Alison</t>
         </is>
       </c>
-      <c r="U345" t="inlineStr">
+      <c r="X345" t="inlineStr">
         <is>
           <t>38440</t>
         </is>
@@ -20412,7 +20442,7 @@
           <t>RANKIN Georgia</t>
         </is>
       </c>
-      <c r="U346" t="inlineStr">
+      <c r="X346" t="inlineStr">
         <is>
           <t>38435</t>
         </is>
@@ -20470,7 +20500,7 @@
           <t>KOZOROG Alja</t>
         </is>
       </c>
-      <c r="U347" t="inlineStr">
+      <c r="X347" t="inlineStr">
         <is>
           <t>39986</t>
         </is>
@@ -20528,7 +20558,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U348" t="inlineStr">
+      <c r="X348" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -20586,7 +20616,7 @@
           <t>GLEJTEKOVA Simona</t>
         </is>
       </c>
-      <c r="U349" t="inlineStr">
+      <c r="X349" t="inlineStr">
         <is>
           <t>55166</t>
         </is>
@@ -20644,7 +20674,7 @@
           <t>TIXIER Cecile</t>
         </is>
       </c>
-      <c r="U350" t="inlineStr">
+      <c r="X350" t="inlineStr">
         <is>
           <t>35687</t>
         </is>
@@ -20702,7 +20732,7 @@
           <t>BIZJAK Nina</t>
         </is>
       </c>
-      <c r="U351" t="inlineStr">
+      <c r="X351" t="inlineStr">
         <is>
           <t>39984</t>
         </is>
@@ -20760,7 +20790,7 @@
           <t>WERATSCHNIG Nadine</t>
         </is>
       </c>
-      <c r="U352" t="inlineStr">
+      <c r="X352" t="inlineStr">
         <is>
           <t>41613</t>
         </is>
@@ -20818,7 +20848,7 @@
           <t>MATULKOVA Jana</t>
         </is>
       </c>
-      <c r="U353" t="inlineStr">
+      <c r="X353" t="inlineStr">
         <is>
           <t>37274</t>
         </is>
@@ -20876,7 +20906,7 @@
           <t>JACQUET Claire</t>
         </is>
       </c>
-      <c r="U354" t="inlineStr">
+      <c r="X354" t="inlineStr">
         <is>
           <t>35684</t>
         </is>
@@ -20934,7 +20964,7 @@
           <t>HENRY Margaux</t>
         </is>
       </c>
-      <c r="U355" t="inlineStr">
+      <c r="X355" t="inlineStr">
         <is>
           <t>51995</t>
         </is>
@@ -20992,7 +21022,7 @@
           <t>LAZKANO Miren</t>
         </is>
       </c>
-      <c r="U356" t="inlineStr">
+      <c r="X356" t="inlineStr">
         <is>
           <t>35748</t>
         </is>
@@ -21103,7 +21133,7 @@
           <t>WOLFFHARDT Viktoria</t>
         </is>
       </c>
-      <c r="U358" t="inlineStr">
+      <c r="X358" t="inlineStr">
         <is>
           <t>35303</t>
         </is>
@@ -21161,7 +21191,7 @@
           <t>JANCOVA Monika</t>
         </is>
       </c>
-      <c r="U359" t="inlineStr">
+      <c r="X359" t="inlineStr">
         <is>
           <t>36015</t>
         </is>
@@ -21219,7 +21249,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U360" t="inlineStr">
+      <c r="X360" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -21277,7 +21307,7 @@
           <t>GIBSON Eilidh</t>
         </is>
       </c>
-      <c r="U361" t="inlineStr">
+      <c r="X361" t="inlineStr">
         <is>
           <t>36708</t>
         </is>
@@ -21335,7 +21365,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U362" t="inlineStr">
+      <c r="X362" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -21393,7 +21423,7 @@
           <t>VILARRUBLA Nuria</t>
         </is>
       </c>
-      <c r="U363" t="inlineStr">
+      <c r="X363" t="inlineStr">
         <is>
           <t>35746</t>
         </is>
@@ -21451,7 +21481,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U364" t="inlineStr">
+      <c r="X364" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -21509,7 +21539,7 @@
           <t>WEGER Jakob</t>
         </is>
       </c>
-      <c r="U365" t="inlineStr">
+      <c r="X365" t="inlineStr">
         <is>
           <t>54909</t>
         </is>
@@ -21567,7 +21597,7 @@
           <t>PETERLIN Janos</t>
         </is>
       </c>
-      <c r="U366" t="inlineStr">
+      <c r="X366" t="inlineStr">
         <is>
           <t>36268</t>
         </is>
@@ -21625,7 +21655,7 @@
           <t>GILBERT Callum</t>
         </is>
       </c>
-      <c r="U367" t="inlineStr">
+      <c r="X367" t="inlineStr">
         <is>
           <t>42090</t>
         </is>
@@ -21683,7 +21713,7 @@
           <t>HILGERT Lubos</t>
         </is>
       </c>
-      <c r="U368" t="inlineStr">
+      <c r="X368" t="inlineStr">
         <is>
           <t>35032</t>
         </is>
@@ -21794,7 +21824,7 @@
           <t>DAILLE Etienne</t>
         </is>
       </c>
-      <c r="U370" t="inlineStr">
+      <c r="X370" t="inlineStr">
         <is>
           <t>35308</t>
         </is>
@@ -21852,7 +21882,7 @@
           <t>LAUNAY Antoine</t>
         </is>
       </c>
-      <c r="U371" t="inlineStr">
+      <c r="X371" t="inlineStr">
         <is>
           <t>68776</t>
         </is>
@@ -21910,7 +21940,7 @@
           <t>BRUS Simon</t>
         </is>
       </c>
-      <c r="U372" t="inlineStr">
+      <c r="X372" t="inlineStr">
         <is>
           <t>39076</t>
         </is>
@@ -21968,7 +21998,7 @@
           <t>OSCHMAUTZ Felix</t>
         </is>
       </c>
-      <c r="U373" t="inlineStr">
+      <c r="X373" t="inlineStr">
         <is>
           <t>51856</t>
         </is>
@@ -22026,7 +22056,7 @@
           <t>SRABOTNIK Martin</t>
         </is>
       </c>
-      <c r="U374" t="inlineStr">
+      <c r="X374" t="inlineStr">
         <is>
           <t>39080</t>
         </is>
@@ -22084,7 +22114,7 @@
           <t>LEE EDWARDS Ciaran</t>
         </is>
       </c>
-      <c r="U375" t="inlineStr">
+      <c r="X375" t="inlineStr">
         <is>
           <t>35614</t>
         </is>
@@ -22142,7 +22172,7 @@
           <t>MAXEINER Tim</t>
         </is>
       </c>
-      <c r="U376" t="inlineStr">
+      <c r="X376" t="inlineStr">
         <is>
           <t>35117</t>
         </is>
@@ -22200,7 +22230,7 @@
           <t>BOECKELMANN Paul</t>
         </is>
       </c>
-      <c r="U377" t="inlineStr">
+      <c r="X377" t="inlineStr">
         <is>
           <t>35118</t>
         </is>
@@ -22258,7 +22288,7 @@
           <t>BUTCHER Finn</t>
         </is>
       </c>
-      <c r="U378" t="inlineStr">
+      <c r="X378" t="inlineStr">
         <is>
           <t>36663</t>
         </is>
@@ -22369,7 +22399,7 @@
           <t>POWELL Richard</t>
         </is>
       </c>
-      <c r="U380" t="inlineStr">
+      <c r="X380" t="inlineStr">
         <is>
           <t>36444</t>
         </is>
@@ -22427,7 +22457,7 @@
           <t>MEGLIC Jure</t>
         </is>
       </c>
-      <c r="U381" t="inlineStr">
+      <c r="X381" t="inlineStr">
         <is>
           <t>35590</t>
         </is>
@@ -22485,7 +22515,7 @@
           <t>CHIARELLO Gelindo</t>
         </is>
       </c>
-      <c r="U382" t="inlineStr">
+      <c r="X382" t="inlineStr">
         <is>
           <t>39956</t>
         </is>
@@ -22543,7 +22573,7 @@
           <t>OHRSTROM Isak</t>
         </is>
       </c>
-      <c r="U383" t="inlineStr">
+      <c r="X383" t="inlineStr">
         <is>
           <t>35101</t>
         </is>
@@ -22601,7 +22631,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U384" t="inlineStr">
+      <c r="X384" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -22659,7 +22689,7 @@
           <t>DOBY Mathieu</t>
         </is>
       </c>
-      <c r="U385" t="inlineStr">
+      <c r="X385" t="inlineStr">
         <is>
           <t>35292</t>
         </is>
@@ -22717,7 +22747,7 @@
           <t>MOLMENTI Daniele</t>
         </is>
       </c>
-      <c r="U386" t="inlineStr">
+      <c r="X386" t="inlineStr">
         <is>
           <t>42017</t>
         </is>
@@ -22775,7 +22805,7 @@
           <t>DRAPER Warwick</t>
         </is>
       </c>
-      <c r="U387" t="inlineStr">
+      <c r="X387" t="inlineStr">
         <is>
           <t>36536</t>
         </is>
@@ -22833,7 +22863,7 @@
           <t>ALBREHT Martin</t>
         </is>
       </c>
-      <c r="U388" t="inlineStr">
+      <c r="X388" t="inlineStr">
         <is>
           <t>36898</t>
         </is>
@@ -22891,7 +22921,7 @@
           <t>HUJSA Matus</t>
         </is>
       </c>
-      <c r="U389" t="inlineStr">
+      <c r="X389" t="inlineStr">
         <is>
           <t>35503</t>
         </is>
@@ -22949,7 +22979,7 @@
           <t>BOURLIAUD Pierre</t>
         </is>
       </c>
-      <c r="U390" t="inlineStr">
+      <c r="X390" t="inlineStr">
         <is>
           <t>35230</t>
         </is>
@@ -23007,7 +23037,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U391" t="inlineStr">
+      <c r="X391" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -23065,7 +23095,7 @@
           <t>FORBES-CRYANS Bradley</t>
         </is>
       </c>
-      <c r="U392" t="inlineStr">
+      <c r="X392" t="inlineStr">
         <is>
           <t>36513</t>
         </is>
@@ -23123,7 +23153,7 @@
           <t>LEITNER Mario</t>
         </is>
       </c>
-      <c r="U393" t="inlineStr">
+      <c r="X393" t="inlineStr">
         <is>
           <t>35546</t>
         </is>
@@ -23181,7 +23211,7 @@
           <t>BERSINGER Thomas</t>
         </is>
       </c>
-      <c r="U394" t="inlineStr">
+      <c r="X394" t="inlineStr">
         <is>
           <t>35228</t>
         </is>
@@ -23239,7 +23269,7 @@
           <t>BIAZIZZO Mathieu</t>
         </is>
       </c>
-      <c r="U395" t="inlineStr">
+      <c r="X395" t="inlineStr">
         <is>
           <t>35484</t>
         </is>
@@ -23297,7 +23327,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U396" t="inlineStr">
+      <c r="X396" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -23355,7 +23385,7 @@
           <t>GRIMM Alexander</t>
         </is>
       </c>
-      <c r="U397" t="inlineStr">
+      <c r="X397" t="inlineStr">
         <is>
           <t>35112</t>
         </is>
@@ -23413,7 +23443,7 @@
           <t>PRINDIS Vit</t>
         </is>
       </c>
-      <c r="U398" t="inlineStr">
+      <c r="X398" t="inlineStr">
         <is>
           <t>35065</t>
         </is>
@@ -23471,7 +23501,7 @@
           <t>TUNKA Ondrej</t>
         </is>
       </c>
-      <c r="U399" t="inlineStr">
+      <c r="X399" t="inlineStr">
         <is>
           <t>35947</t>
         </is>
@@ -23529,7 +23559,7 @@
           <t>CRESPO Joan</t>
         </is>
       </c>
-      <c r="U400" t="inlineStr">
+      <c r="X400" t="inlineStr">
         <is>
           <t>35749</t>
         </is>
@@ -23587,7 +23617,7 @@
           <t>HRADILEK Vavrinec</t>
         </is>
       </c>
-      <c r="U401" t="inlineStr">
+      <c r="X401" t="inlineStr">
         <is>
           <t>35031</t>
         </is>
@@ -23645,7 +23675,7 @@
           <t>HALCIN Martin</t>
         </is>
       </c>
-      <c r="U402" t="inlineStr">
+      <c r="X402" t="inlineStr">
         <is>
           <t>35355</t>
         </is>
@@ -23703,7 +23733,7 @@
           <t>SCHUBERT Sebastian</t>
         </is>
       </c>
-      <c r="U403" t="inlineStr">
+      <c r="X403" t="inlineStr">
         <is>
           <t>35114</t>
         </is>
@@ -23761,7 +23791,7 @@
           <t>RENIA Benjamin</t>
         </is>
       </c>
-      <c r="U404" t="inlineStr">
+      <c r="X404" t="inlineStr">
         <is>
           <t>35407</t>
         </is>
@@ -23829,7 +23859,7 @@
           <t>KOECHLIN Thomas</t>
         </is>
       </c>
-      <c r="U405" t="inlineStr">
+      <c r="X405" t="inlineStr">
         <is>
           <t>35419</t>
         </is>
@@ -23897,7 +23927,7 @@
           <t>FOULON Kilian</t>
         </is>
       </c>
-      <c r="U406" t="inlineStr">
+      <c r="X406" t="inlineStr">
         <is>
           <t>35602</t>
         </is>
@@ -23965,7 +23995,7 @@
           <t>RAK Tomas</t>
         </is>
       </c>
-      <c r="U407" t="inlineStr">
+      <c r="X407" t="inlineStr">
         <is>
           <t>35056</t>
         </is>
@@ -24033,7 +24063,7 @@
           <t>LENARCIC Jure</t>
         </is>
       </c>
-      <c r="U408" t="inlineStr">
+      <c r="X408" t="inlineStr">
         <is>
           <t>36259</t>
         </is>
@@ -24101,7 +24131,7 @@
           <t>BERCIC Anze</t>
         </is>
       </c>
-      <c r="U409" t="inlineStr">
+      <c r="X409" t="inlineStr">
         <is>
           <t>36253</t>
         </is>
@@ -24169,7 +24199,7 @@
           <t>TILLARD Pierre-Antoine</t>
         </is>
       </c>
-      <c r="U410" t="inlineStr">
+      <c r="X410" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
@@ -24237,7 +24267,7 @@
           <t>COLAZINGARI Roberto</t>
         </is>
       </c>
-      <c r="U411" t="inlineStr">
+      <c r="X411" t="inlineStr">
         <is>
           <t>35223</t>
         </is>
@@ -24305,7 +24335,7 @@
           <t>THOMAS Martin</t>
         </is>
       </c>
-      <c r="U412" t="inlineStr">
+      <c r="X412" t="inlineStr">
         <is>
           <t>35412</t>
         </is>
@@ -24373,7 +24403,7 @@
           <t>MARTIKAN Michal</t>
         </is>
       </c>
-      <c r="U413" t="inlineStr">
+      <c r="X413" t="inlineStr">
         <is>
           <t>35365</t>
         </is>
@@ -24441,7 +24471,7 @@
           <t>JANE Michal</t>
         </is>
       </c>
-      <c r="U414" t="inlineStr">
+      <c r="X414" t="inlineStr">
         <is>
           <t>35059</t>
         </is>
@@ -24509,7 +24539,7 @@
           <t>HENRY Margaux</t>
         </is>
       </c>
-      <c r="U415" t="inlineStr">
+      <c r="X415" t="inlineStr">
         <is>
           <t>51995</t>
         </is>
@@ -24577,7 +24607,7 @@
           <t>OLAZABAL Klara</t>
         </is>
       </c>
-      <c r="U416" t="inlineStr">
+      <c r="X416" t="inlineStr">
         <is>
           <t>43985</t>
         </is>
@@ -24645,7 +24675,7 @@
           <t>GLEJTEKOVA Simona</t>
         </is>
       </c>
-      <c r="U417" t="inlineStr">
+      <c r="X417" t="inlineStr">
         <is>
           <t>55166</t>
         </is>
@@ -24776,7 +24806,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U419" t="inlineStr">
+      <c r="X419" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -24844,7 +24874,7 @@
           <t>JANCOVA Monika</t>
         </is>
       </c>
-      <c r="U420" t="inlineStr">
+      <c r="X420" t="inlineStr">
         <is>
           <t>36015</t>
         </is>
@@ -24912,7 +24942,7 @@
           <t>GIBSON Eilidh</t>
         </is>
       </c>
-      <c r="U421" t="inlineStr">
+      <c r="X421" t="inlineStr">
         <is>
           <t>36708</t>
         </is>
@@ -24980,7 +25010,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U422" t="inlineStr">
+      <c r="X422" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -25048,7 +25078,7 @@
           <t>JACQUET Claire</t>
         </is>
       </c>
-      <c r="U423" t="inlineStr">
+      <c r="X423" t="inlineStr">
         <is>
           <t>35684</t>
         </is>
@@ -25116,7 +25146,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U424" t="inlineStr">
+      <c r="X424" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -25184,7 +25214,7 @@
           <t>DE GENNARO Giovanni</t>
         </is>
       </c>
-      <c r="U425" t="inlineStr">
+      <c r="X425" t="inlineStr">
         <is>
           <t>35244</t>
         </is>
@@ -25252,7 +25282,7 @@
           <t>MOLMENTI Daniele</t>
         </is>
       </c>
-      <c r="U426" t="inlineStr">
+      <c r="X426" t="inlineStr">
         <is>
           <t>42017</t>
         </is>
@@ -25320,7 +25350,7 @@
           <t>FORBES-CRYANS Bradley</t>
         </is>
       </c>
-      <c r="U427" t="inlineStr">
+      <c r="X427" t="inlineStr">
         <is>
           <t>36513</t>
         </is>
@@ -25388,7 +25418,7 @@
           <t>TUNKA Ondrej</t>
         </is>
       </c>
-      <c r="U428" t="inlineStr">
+      <c r="X428" t="inlineStr">
         <is>
           <t>35947</t>
         </is>
@@ -25456,7 +25486,7 @@
           <t>DAILLE Etienne</t>
         </is>
       </c>
-      <c r="U429" t="inlineStr">
+      <c r="X429" t="inlineStr">
         <is>
           <t>35308</t>
         </is>
@@ -25524,7 +25554,7 @@
           <t>BERSINGER Thomas</t>
         </is>
       </c>
-      <c r="U430" t="inlineStr">
+      <c r="X430" t="inlineStr">
         <is>
           <t>35228</t>
         </is>
@@ -25592,7 +25622,7 @@
           <t>DOBY Mathieu</t>
         </is>
       </c>
-      <c r="U431" t="inlineStr">
+      <c r="X431" t="inlineStr">
         <is>
           <t>35292</t>
         </is>
@@ -25660,7 +25690,7 @@
           <t>HERNANZ Samuel</t>
         </is>
       </c>
-      <c r="U432" t="inlineStr">
+      <c r="X432" t="inlineStr">
         <is>
           <t>35786</t>
         </is>
@@ -25728,7 +25758,7 @@
           <t>POPIELA Dariusz</t>
         </is>
       </c>
-      <c r="U433" t="inlineStr">
+      <c r="X433" t="inlineStr">
         <is>
           <t>35096</t>
         </is>
@@ -25796,7 +25826,7 @@
           <t>HALCIN Martin</t>
         </is>
       </c>
-      <c r="U434" t="inlineStr">
+      <c r="X434" t="inlineStr">
         <is>
           <t>35355</t>
         </is>
@@ -25854,7 +25884,7 @@
           <t>SABATTINI Chiara</t>
         </is>
       </c>
-      <c r="U435" t="inlineStr">
+      <c r="X435" t="inlineStr">
         <is>
           <t>35219</t>
         </is>
@@ -26018,7 +26048,7 @@
           <t>FOX Noemie</t>
         </is>
       </c>
-      <c r="U438" t="inlineStr">
+      <c r="X438" t="inlineStr">
         <is>
           <t>44812</t>
         </is>
@@ -26076,7 +26106,7 @@
           <t>HILGERTOVA Amalie</t>
         </is>
       </c>
-      <c r="U439" t="inlineStr">
+      <c r="X439" t="inlineStr">
         <is>
           <t>36113</t>
         </is>
@@ -26134,7 +26164,7 @@
           <t>GRAILLE Solene</t>
         </is>
       </c>
-      <c r="U440" t="inlineStr">
+      <c r="X440" t="inlineStr">
         <is>
           <t>36211</t>
         </is>
@@ -26245,7 +26275,7 @@
           <t>US Viktoriia</t>
         </is>
       </c>
-      <c r="U442" t="inlineStr">
+      <c r="X442" t="inlineStr">
         <is>
           <t>35528</t>
         </is>
@@ -26303,7 +26333,7 @@
           <t>GROENEVELD Jessica</t>
         </is>
       </c>
-      <c r="U443" t="inlineStr">
+      <c r="X443" t="inlineStr">
         <is>
           <t>35542</t>
         </is>
@@ -26361,7 +26391,7 @@
           <t>KALISKA Elena</t>
         </is>
       </c>
-      <c r="U444" t="inlineStr">
+      <c r="X444" t="inlineStr">
         <is>
           <t>35366</t>
         </is>
@@ -26419,7 +26449,7 @@
           <t>NEVARILOVA Kristina</t>
         </is>
       </c>
-      <c r="U445" t="inlineStr">
+      <c r="X445" t="inlineStr">
         <is>
           <t>35467</t>
         </is>
@@ -26530,7 +26560,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U447" t="inlineStr">
+      <c r="X447" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -26588,7 +26618,7 @@
           <t>WOODS Kimberley</t>
         </is>
       </c>
-      <c r="U448" t="inlineStr">
+      <c r="X448" t="inlineStr">
         <is>
           <t>35650</t>
         </is>
@@ -26646,7 +26676,7 @@
           <t>FRANKLIN Mallory</t>
         </is>
       </c>
-      <c r="U449" t="inlineStr">
+      <c r="X449" t="inlineStr">
         <is>
           <t>35615</t>
         </is>
@@ -26704,7 +26734,7 @@
           <t>MANGIN Estelle</t>
         </is>
       </c>
-      <c r="U450" t="inlineStr">
+      <c r="X450" t="inlineStr">
         <is>
           <t>35670</t>
         </is>
@@ -26762,7 +26792,7 @@
           <t>WEGMAN Martina</t>
         </is>
       </c>
-      <c r="U451" t="inlineStr">
+      <c r="X451" t="inlineStr">
         <is>
           <t>35345</t>
         </is>
@@ -26820,7 +26850,7 @@
           <t>LEITNER Lisa</t>
         </is>
       </c>
-      <c r="U452" t="inlineStr">
+      <c r="X452" t="inlineStr">
         <is>
           <t>35305</t>
         </is>
@@ -26878,7 +26908,7 @@
           <t>VOJTOVA Veronika</t>
         </is>
       </c>
-      <c r="U453" t="inlineStr">
+      <c r="X453" t="inlineStr">
         <is>
           <t>35945</t>
         </is>
@@ -26936,7 +26966,7 @@
           <t>TERCELJ Eva</t>
         </is>
       </c>
-      <c r="U454" t="inlineStr">
+      <c r="X454" t="inlineStr">
         <is>
           <t>36263</t>
         </is>
@@ -26994,7 +27024,7 @@
           <t>LI Lu</t>
         </is>
       </c>
-      <c r="U455" t="inlineStr">
+      <c r="X455" t="inlineStr">
         <is>
           <t>37086</t>
         </is>
@@ -27052,7 +27082,7 @@
           <t>OBLINGER-PETERS Violetta</t>
         </is>
       </c>
-      <c r="U456" t="inlineStr">
+      <c r="X456" t="inlineStr">
         <is>
           <t>35289</t>
         </is>
@@ -27110,7 +27140,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U457" t="inlineStr">
+      <c r="X457" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -27168,7 +27198,7 @@
           <t>BOUZIDI Carole</t>
         </is>
       </c>
-      <c r="U458" t="inlineStr">
+      <c r="X458" t="inlineStr">
         <is>
           <t>35231</t>
         </is>
@@ -27226,7 +27256,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U459" t="inlineStr">
+      <c r="X459" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -27284,7 +27314,7 @@
           <t>HILGERTOVA Stepanka</t>
         </is>
       </c>
-      <c r="U460" t="inlineStr">
+      <c r="X460" t="inlineStr">
         <is>
           <t>35035</t>
         </is>
@@ -27342,7 +27372,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U461" t="inlineStr">
+      <c r="X461" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -27400,7 +27430,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U462" t="inlineStr">
+      <c r="X462" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -27458,7 +27488,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U463" t="inlineStr">
+      <c r="X463" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -27516,7 +27546,7 @@
           <t>GOIKOETXEA Irati</t>
         </is>
       </c>
-      <c r="U464" t="inlineStr">
+      <c r="X464" t="inlineStr">
         <is>
           <t>35761</t>
         </is>
@@ -27574,7 +27604,7 @@
           <t>MARTINEZ Marta</t>
         </is>
       </c>
-      <c r="U465" t="inlineStr">
+      <c r="X465" t="inlineStr">
         <is>
           <t>35760</t>
         </is>
@@ -27632,7 +27662,7 @@
           <t>GUIET Pauline</t>
         </is>
       </c>
-      <c r="U466" t="inlineStr">
+      <c r="X466" t="inlineStr">
         <is>
           <t>35493</t>
         </is>
@@ -27690,7 +27720,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U467" t="inlineStr">
+      <c r="X467" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -27753,12 +27783,12 @@
           <t>OLIVEIRA Anderson</t>
         </is>
       </c>
-      <c r="U468" t="inlineStr">
+      <c r="X468" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
       </c>
-      <c r="V468" t="inlineStr">
+      <c r="Y468" t="inlineStr">
         <is>
           <t>38020</t>
         </is>
@@ -27821,12 +27851,12 @@
           <t>VIEIRA Cassiano</t>
         </is>
       </c>
-      <c r="U469" t="inlineStr">
+      <c r="X469" t="inlineStr">
         <is>
           <t>42977</t>
         </is>
       </c>
-      <c r="V469" t="inlineStr">
+      <c r="Y469" t="inlineStr">
         <is>
           <t>42976</t>
         </is>
@@ -27889,12 +27919,12 @@
           <t>KASPAR Albert</t>
         </is>
       </c>
-      <c r="U470" t="inlineStr">
+      <c r="X470" t="inlineStr">
         <is>
           <t>42012</t>
         </is>
       </c>
-      <c r="V470" t="inlineStr">
+      <c r="Y470" t="inlineStr">
         <is>
           <t>42013</t>
         </is>
@@ -27957,12 +27987,12 @@
           <t>MUELLER Kevin</t>
         </is>
       </c>
-      <c r="U471" t="inlineStr">
+      <c r="X471" t="inlineStr">
         <is>
           <t>35148</t>
         </is>
       </c>
-      <c r="V471" t="inlineStr">
+      <c r="Y471" t="inlineStr">
         <is>
           <t>35149</t>
         </is>
@@ -28025,12 +28055,12 @@
           <t>KERVELLA Loic</t>
         </is>
       </c>
-      <c r="U472" t="inlineStr">
+      <c r="X472" t="inlineStr">
         <is>
           <t>35671</t>
         </is>
       </c>
-      <c r="V472" t="inlineStr">
+      <c r="Y472" t="inlineStr">
         <is>
           <t>35672</t>
         </is>
@@ -28093,12 +28123,12 @@
           <t>DENG Xiao</t>
         </is>
       </c>
-      <c r="U473" t="inlineStr">
+      <c r="X473" t="inlineStr">
         <is>
           <t>42239</t>
         </is>
       </c>
-      <c r="V473" t="inlineStr">
+      <c r="Y473" t="inlineStr">
         <is>
           <t>42240</t>
         </is>
@@ -28161,12 +28191,12 @@
           <t>PEREZ Jesus</t>
         </is>
       </c>
-      <c r="U474" t="inlineStr">
+      <c r="X474" t="inlineStr">
         <is>
           <t>35757</t>
         </is>
       </c>
-      <c r="V474" t="inlineStr">
+      <c r="Y474" t="inlineStr">
         <is>
           <t>36091</t>
         </is>
@@ -28229,12 +28259,12 @@
           <t>JANE Jakub</t>
         </is>
       </c>
-      <c r="U475" t="inlineStr">
+      <c r="X475" t="inlineStr">
         <is>
           <t>35060</t>
         </is>
       </c>
-      <c r="V475" t="inlineStr">
+      <c r="Y475" t="inlineStr">
         <is>
           <t>35061</t>
         </is>
@@ -28297,12 +28327,12 @@
           <t>BATIK Jan</t>
         </is>
       </c>
-      <c r="U476" t="inlineStr">
+      <c r="X476" t="inlineStr">
         <is>
           <t>35368</t>
         </is>
       </c>
-      <c r="V476" t="inlineStr">
+      <c r="Y476" t="inlineStr">
         <is>
           <t>35367</t>
         </is>
@@ -28365,12 +28395,12 @@
           <t>CHEN Jin</t>
         </is>
       </c>
-      <c r="U477" t="inlineStr">
+      <c r="X477" t="inlineStr">
         <is>
           <t>42237</t>
         </is>
       </c>
-      <c r="V477" t="inlineStr">
+      <c r="Y477" t="inlineStr">
         <is>
           <t>42238</t>
         </is>
@@ -28433,12 +28463,12 @@
           <t>FERRARI Niccolo</t>
         </is>
       </c>
-      <c r="U478" t="inlineStr">
+      <c r="X478" t="inlineStr">
         <is>
           <t>35497</t>
         </is>
       </c>
-      <c r="V478" t="inlineStr">
+      <c r="Y478" t="inlineStr">
         <is>
           <t>35498</t>
         </is>
@@ -28501,12 +28531,12 @@
           <t>HOCHSCHORNER Peter</t>
         </is>
       </c>
-      <c r="U479" t="inlineStr">
+      <c r="X479" t="inlineStr">
         <is>
           <t>35356</t>
         </is>
       </c>
-      <c r="V479" t="inlineStr">
+      <c r="Y479" t="inlineStr">
         <is>
           <t>35357</t>
         </is>
@@ -28569,12 +28599,12 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U480" t="inlineStr">
+      <c r="X480" t="inlineStr">
         <is>
           <t>35145</t>
         </is>
       </c>
-      <c r="V480" t="inlineStr">
+      <c r="Y480" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -28637,12 +28667,12 @@
           <t>BISO Hugo</t>
         </is>
       </c>
-      <c r="U481" t="inlineStr">
+      <c r="X481" t="inlineStr">
         <is>
           <t>35403</t>
         </is>
       </c>
-      <c r="V481" t="inlineStr">
+      <c r="Y481" t="inlineStr">
         <is>
           <t>35229</t>
         </is>
@@ -28705,12 +28735,12 @@
           <t>CAILHOL Hugo</t>
         </is>
       </c>
-      <c r="U482" t="inlineStr">
+      <c r="X482" t="inlineStr">
         <is>
           <t>35476</t>
         </is>
       </c>
-      <c r="V482" t="inlineStr">
+      <c r="Y482" t="inlineStr">
         <is>
           <t>35491</t>
         </is>
@@ -28773,12 +28803,12 @@
           <t>BECKER Thomas</t>
         </is>
       </c>
-      <c r="U483" t="inlineStr">
+      <c r="X483" t="inlineStr">
         <is>
           <t>35139</t>
         </is>
       </c>
-      <c r="V483" t="inlineStr">
+      <c r="Y483" t="inlineStr">
         <is>
           <t>35143</t>
         </is>
@@ -28841,12 +28871,12 @@
           <t>LE RUYET Edern</t>
         </is>
       </c>
-      <c r="U484" t="inlineStr">
+      <c r="X484" t="inlineStr">
         <is>
           <t>35413</t>
         </is>
       </c>
-      <c r="V484" t="inlineStr">
+      <c r="Y484" t="inlineStr">
         <is>
           <t>35379</t>
         </is>
@@ -28914,7 +28944,7 @@
           <t>SCHORNBERG Jasmin</t>
         </is>
       </c>
-      <c r="U485" t="inlineStr">
+      <c r="X485" t="inlineStr">
         <is>
           <t>35206</t>
         </is>
@@ -28982,7 +29012,7 @@
           <t>MANGIN Estelle</t>
         </is>
       </c>
-      <c r="U486" t="inlineStr">
+      <c r="X486" t="inlineStr">
         <is>
           <t>35670</t>
         </is>
@@ -29050,7 +29080,7 @@
           <t>HORN Stefanie</t>
         </is>
       </c>
-      <c r="U487" t="inlineStr">
+      <c r="X487" t="inlineStr">
         <is>
           <t>38417</t>
         </is>
@@ -29118,7 +29148,7 @@
           <t>SATILA Ana</t>
         </is>
       </c>
-      <c r="U488" t="inlineStr">
+      <c r="X488" t="inlineStr">
         <is>
           <t>35327</t>
         </is>
@@ -29186,7 +29216,7 @@
           <t>KUHNLE Corinna</t>
         </is>
       </c>
-      <c r="U489" t="inlineStr">
+      <c r="X489" t="inlineStr">
         <is>
           <t>35282</t>
         </is>
@@ -29254,7 +29284,7 @@
           <t>FOX Jessica</t>
         </is>
       </c>
-      <c r="U490" t="inlineStr">
+      <c r="X490" t="inlineStr">
         <is>
           <t>36526</t>
         </is>
@@ -29322,7 +29352,7 @@
           <t>LI Lu</t>
         </is>
       </c>
-      <c r="U491" t="inlineStr">
+      <c r="X491" t="inlineStr">
         <is>
           <t>37086</t>
         </is>
@@ -29453,7 +29483,7 @@
           <t>DUKATOVA Jana</t>
         </is>
       </c>
-      <c r="U493" t="inlineStr">
+      <c r="X493" t="inlineStr">
         <is>
           <t>35354</t>
         </is>
@@ -29521,7 +29551,7 @@
           <t>FUNK Ricarda</t>
         </is>
       </c>
-      <c r="U494" t="inlineStr">
+      <c r="X494" t="inlineStr">
         <is>
           <t>35122</t>
         </is>
@@ -29594,12 +29624,12 @@
           <t>MUELLER Kevin</t>
         </is>
       </c>
-      <c r="U495" t="inlineStr">
+      <c r="X495" t="inlineStr">
         <is>
           <t>35148</t>
         </is>
       </c>
-      <c r="V495" t="inlineStr">
+      <c r="Y495" t="inlineStr">
         <is>
           <t>35149</t>
         </is>
@@ -29672,12 +29702,12 @@
           <t>DENG Xiao</t>
         </is>
       </c>
-      <c r="U496" t="inlineStr">
+      <c r="X496" t="inlineStr">
         <is>
           <t>42239</t>
         </is>
       </c>
-      <c r="V496" t="inlineStr">
+      <c r="Y496" t="inlineStr">
         <is>
           <t>42240</t>
         </is>
@@ -29750,12 +29780,12 @@
           <t>CAILHOL Hugo</t>
         </is>
       </c>
-      <c r="U497" t="inlineStr">
+      <c r="X497" t="inlineStr">
         <is>
           <t>35476</t>
         </is>
       </c>
-      <c r="V497" t="inlineStr">
+      <c r="Y497" t="inlineStr">
         <is>
           <t>35491</t>
         </is>
@@ -29828,12 +29858,12 @@
           <t>PEREZ Jesus</t>
         </is>
       </c>
-      <c r="U498" t="inlineStr">
+      <c r="X498" t="inlineStr">
         <is>
           <t>35757</t>
         </is>
       </c>
-      <c r="V498" t="inlineStr">
+      <c r="Y498" t="inlineStr">
         <is>
           <t>36091</t>
         </is>
@@ -29906,12 +29936,12 @@
           <t>JANE Jakub</t>
         </is>
       </c>
-      <c r="U499" t="inlineStr">
+      <c r="X499" t="inlineStr">
         <is>
           <t>35060</t>
         </is>
       </c>
-      <c r="V499" t="inlineStr">
+      <c r="Y499" t="inlineStr">
         <is>
           <t>35061</t>
         </is>
@@ -29984,12 +30014,12 @@
           <t>OLIVEIRA Anderson</t>
         </is>
       </c>
-      <c r="U500" t="inlineStr">
+      <c r="X500" t="inlineStr">
         <is>
           <t>38018</t>
         </is>
       </c>
-      <c r="V500" t="inlineStr">
+      <c r="Y500" t="inlineStr">
         <is>
           <t>38020</t>
         </is>
@@ -30062,12 +30092,12 @@
           <t>BETTGE Nico</t>
         </is>
       </c>
-      <c r="U501" t="inlineStr">
+      <c r="X501" t="inlineStr">
         <is>
           <t>35145</t>
         </is>
       </c>
-      <c r="V501" t="inlineStr">
+      <c r="Y501" t="inlineStr">
         <is>
           <t>35133</t>
         </is>
@@ -30140,12 +30170,12 @@
           <t>KERVELLA Loic</t>
         </is>
       </c>
-      <c r="U502" t="inlineStr">
+      <c r="X502" t="inlineStr">
         <is>
           <t>35671</t>
         </is>
       </c>
-      <c r="V502" t="inlineStr">
+      <c r="Y502" t="inlineStr">
         <is>
           <t>35672</t>
         </is>
@@ -30218,12 +30248,12 @@
           <t>HOCHSCHORNER Peter</t>
         </is>
       </c>
-      <c r="U503" t="inlineStr">
+      <c r="X503" t="inlineStr">
         <is>
           <t>35356</t>
         </is>
       </c>
-      <c r="V503" t="inlineStr">
+      <c r="Y503" t="inlineStr">
         <is>
           <t>35357</t>
         </is>
@@ -30296,12 +30326,12 @@
           <t>BISO Hugo</t>
         </is>
       </c>
-      <c r="U504" t="inlineStr">
+      <c r="X504" t="inlineStr">
         <is>
           <t>35403</t>
         </is>
       </c>
-      <c r="V504" t="inlineStr">
+      <c r="Y504" t="inlineStr">
         <is>
           <t>35229</t>
         </is>

</xml_diff>